<commit_message>
Add design system pages, update home and overview deck
- Design system: DesignSystemLayout, atoms/molecules/index pages, design-system.css
- Home: copy/content updates
- Overview deck: minor update
- CLAUDE.md and PAGES.xlsx: updated inventory

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I16"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="8" min="1" max="1"/>
@@ -503,163 +503,163 @@
       </c>
     </row>
     <row r="2" ht="36" customHeight="1" s="9">
-      <c r="A2" s="11" t="inlineStr">
+      <c r="A2" s="15" t="inlineStr">
         <is>
           <t>Home</t>
         </is>
       </c>
-      <c r="B2" s="11" t="inlineStr">
+      <c r="B2" s="15" t="inlineStr">
         <is>
           <t>https://compoundhealth.io/</t>
         </is>
       </c>
-      <c r="C2" s="11" t="inlineStr">
+      <c r="C2" s="15" t="inlineStr">
         <is>
           <t>/</t>
         </is>
       </c>
-      <c r="D2" s="12" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="E2" s="13" t="inlineStr">
+      <c r="D2" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>Indexed</t>
         </is>
       </c>
-      <c r="F2" s="11" t="inlineStr">
+      <c r="F2" s="15" t="inlineStr">
         <is>
           <t>MainLayout</t>
         </is>
       </c>
-      <c r="G2" s="11" t="inlineStr">
+      <c r="G2" s="15" t="inlineStr">
         <is>
           <t>src/pages/index.astro</t>
         </is>
       </c>
-      <c r="H2" s="11" t="inlineStr">
+      <c r="H2" s="15" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="I2" s="11" t="inlineStr">
+      <c r="I2" s="15" t="inlineStr">
         <is>
           <t>Main marketing landing page</t>
         </is>
       </c>
     </row>
     <row r="3" ht="36" customHeight="1" s="9">
-      <c r="A3" s="11" t="inlineStr">
+      <c r="A3" s="15" t="inlineStr">
         <is>
           <t>Privacy Policy</t>
         </is>
       </c>
-      <c r="B3" s="11" t="inlineStr">
+      <c r="B3" s="15" t="inlineStr">
         <is>
           <t>https://compoundhealth.io/privacy-policy</t>
         </is>
       </c>
-      <c r="C3" s="11" t="inlineStr">
+      <c r="C3" s="15" t="inlineStr">
         <is>
           <t>/privacy-policy</t>
         </is>
       </c>
-      <c r="D3" s="12" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="E3" s="13" t="inlineStr">
+      <c r="D3" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
         <is>
           <t>Indexed</t>
         </is>
       </c>
-      <c r="F3" s="11" t="inlineStr">
+      <c r="F3" s="15" t="inlineStr">
         <is>
           <t>LegalLayout</t>
         </is>
       </c>
-      <c r="G3" s="11" t="inlineStr">
+      <c r="G3" s="15" t="inlineStr">
         <is>
           <t>src/pages/privacy-policy.astro</t>
         </is>
       </c>
-      <c r="H3" s="11" t="inlineStr">
+      <c r="H3" s="15" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="I3" s="11" t="inlineStr">
+      <c r="I3" s="15" t="inlineStr">
         <is>
           <t>Legal — privacy notice</t>
         </is>
       </c>
     </row>
     <row r="4" ht="36" customHeight="1" s="9">
-      <c r="A4" s="11" t="inlineStr">
+      <c r="A4" s="15" t="inlineStr">
         <is>
           <t>Website Terms</t>
         </is>
       </c>
-      <c r="B4" s="11" t="inlineStr">
+      <c r="B4" s="15" t="inlineStr">
         <is>
           <t>https://compoundhealth.io/website-terms</t>
         </is>
       </c>
-      <c r="C4" s="11" t="inlineStr">
+      <c r="C4" s="15" t="inlineStr">
         <is>
           <t>/website-terms</t>
         </is>
       </c>
-      <c r="D4" s="12" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="E4" s="13" t="inlineStr">
+      <c r="D4" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E4" s="17" t="inlineStr">
         <is>
           <t>Indexed</t>
         </is>
       </c>
-      <c r="F4" s="11" t="inlineStr">
+      <c r="F4" s="15" t="inlineStr">
         <is>
           <t>LegalLayout</t>
         </is>
       </c>
-      <c r="G4" s="11" t="inlineStr">
+      <c r="G4" s="15" t="inlineStr">
         <is>
           <t>src/pages/website-terms.astro</t>
         </is>
       </c>
-      <c r="H4" s="11" t="inlineStr">
+      <c r="H4" s="15" t="inlineStr">
         <is>
           <t>2026-04-28</t>
         </is>
       </c>
-      <c r="I4" s="11" t="inlineStr">
+      <c r="I4" s="15" t="inlineStr">
         <is>
           <t>Legal — website terms of use</t>
         </is>
       </c>
     </row>
     <row r="5" ht="36" customHeight="1" s="9">
-      <c r="A5" s="11" t="inlineStr">
+      <c r="A5" s="15" t="inlineStr">
         <is>
           <t>RIA Overview Deck (June)</t>
         </is>
       </c>
-      <c r="B5" s="11" t="inlineStr">
+      <c r="B5" s="15" t="inlineStr">
         <is>
           <t>https://compoundhealth.io/overview-deck-june/</t>
         </is>
       </c>
-      <c r="C5" s="11" t="inlineStr">
+      <c r="C5" s="15" t="inlineStr">
         <is>
           <t>/overview-deck-june/</t>
         </is>
       </c>
-      <c r="D5" s="12" t="inlineStr">
+      <c r="D5" s="16" t="inlineStr">
         <is>
           <t>Live</t>
         </is>
@@ -669,22 +669,22 @@
           <t>Noindex</t>
         </is>
       </c>
-      <c r="F5" s="11" t="inlineStr">
+      <c r="F5" s="15" t="inlineStr">
         <is>
           <t>MainLayout</t>
         </is>
       </c>
-      <c r="G5" s="11" t="inlineStr">
+      <c r="G5" s="15" t="inlineStr">
         <is>
           <t>src/pages/overview-deck-june/index.astro</t>
         </is>
       </c>
-      <c r="H5" s="11" t="inlineStr">
+      <c r="H5" s="15" t="inlineStr">
         <is>
           <t>2026-05-30</t>
         </is>
       </c>
-      <c r="I5" s="11" t="inlineStr">
+      <c r="I5" s="15" t="inlineStr">
         <is>
           <t>Private RIA partnership deck. noindex=true. Also blocked in robots.txt.</t>
         </is>
@@ -1204,6 +1204,147 @@
       <c r="I16" s="15" t="inlineStr">
         <is>
           <t>Dummy author. Posts listed via shared data file.</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="15" t="inlineStr">
+        <is>
+          <t>Design System — Overview</t>
+        </is>
+      </c>
+      <c r="B17" s="15" t="inlineStr">
+        <is>
+          <t>https://compoundhealth.io/design-system</t>
+        </is>
+      </c>
+      <c r="C17" s="15" t="inlineStr">
+        <is>
+          <t>/design-system</t>
+        </is>
+      </c>
+      <c r="D17" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E17" s="17" t="inlineStr">
+        <is>
+          <t>Noindex</t>
+        </is>
+      </c>
+      <c r="F17" s="15" t="inlineStr">
+        <is>
+          <t>DesignSystemLayout</t>
+        </is>
+      </c>
+      <c r="G17" s="15" t="inlineStr">
+        <is>
+          <t>src/pages/design-system/index.astro</t>
+        </is>
+      </c>
+      <c r="H17" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I17" s="15" t="inlineStr">
+        <is>
+          <t>Internal design system overview. Atomic methodology + Finsweet Client-First naming.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="15" t="inlineStr">
+        <is>
+          <t>Design System — Atoms</t>
+        </is>
+      </c>
+      <c r="B18" s="15" t="inlineStr">
+        <is>
+          <t>https://compoundhealth.io/design-system/atoms</t>
+        </is>
+      </c>
+      <c r="C18" s="15" t="inlineStr">
+        <is>
+          <t>/design-system/atoms</t>
+        </is>
+      </c>
+      <c r="D18" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E18" s="17" t="inlineStr">
+        <is>
+          <t>Noindex</t>
+        </is>
+      </c>
+      <c r="F18" s="15" t="inlineStr">
+        <is>
+          <t>DesignSystemLayout</t>
+        </is>
+      </c>
+      <c r="G18" s="15" t="inlineStr">
+        <is>
+          <t>src/pages/design-system/atoms.astro</t>
+        </is>
+      </c>
+      <c r="H18" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I18" s="15" t="inlineStr">
+        <is>
+          <t>Colour, typography, spacing, radii, buttons, badges, eyebrows, dots, avatars, dividers, inputs, links, motion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="15" t="inlineStr">
+        <is>
+          <t>Design System — Molecules</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>https://compoundhealth.io/design-system/molecules</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>/design-system/molecules</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Noindex</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>DesignSystemLayout</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>src/pages/design-system/molecules.astro</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>Step, plan, testimonial, credibility, metric, case stat, case quote, speaker, form field, mobile menu link, author chip, author stack, post card, tag group, breadcrumb, author panel.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Add for-advisors deck; update home copy and design system
- Add /for-advisors private partner deck (noindex) for RIA/family office partnership discussions
- Update home page hero and credibility bar with more accurate, client-data-forward copy
- Replace emoji icons with inline SVGs in home page feature grid
- Update MainLayout default OG description to lead with data ownership positioning
- Design system and blog layout refinements

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/PAGES.xlsx
+++ b/PAGES.xlsx
@@ -442,7 +442,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:I19"/>
+  <dimension ref="A1:I20"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="15" customHeight="0" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="32" customWidth="1" style="8" min="1" max="1"/>
@@ -693,17 +693,17 @@
     <row r="6">
       <c r="A6" s="15" t="inlineStr">
         <is>
-          <t>Blog — Index</t>
+          <t>For Advisors</t>
         </is>
       </c>
       <c r="B6" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog</t>
+          <t>https://compoundhealth.io/for-advisors</t>
         </is>
       </c>
       <c r="C6" s="15" t="inlineStr">
         <is>
-          <t>/blog</t>
+          <t>/for-advisors</t>
         </is>
       </c>
       <c r="D6" s="16" t="inlineStr">
@@ -711,46 +711,46 @@
           <t>Live</t>
         </is>
       </c>
-      <c r="E6" s="17" t="inlineStr">
+      <c r="E6" s="14" t="inlineStr">
         <is>
           <t>Noindex</t>
         </is>
       </c>
       <c r="F6" s="15" t="inlineStr">
         <is>
-          <t>BlogLayout</t>
+          <t>MainLayout</t>
         </is>
       </c>
       <c r="G6" s="15" t="inlineStr">
         <is>
-          <t>src/pages/blog/index.astro</t>
+          <t>src/pages/for-advisors.astro</t>
         </is>
       </c>
       <c r="H6" s="15" t="inlineStr">
         <is>
-          <t>2026-06-02</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="I6" s="15" t="inlineStr">
         <is>
-          <t>Blog landing. Lists all posts with category filter.</t>
+          <t>Private advisor-facing partnership page (item 5). noindex=true; excluded from sitemap. Contains [TO CONFIRM] placeholders for commercial/compliance detail.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="15" t="inlineStr">
         <is>
-          <t>Blog Category — Research</t>
+          <t>Blog — Index</t>
         </is>
       </c>
       <c r="B7" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/category/research</t>
+          <t>https://compoundhealth.io/blog</t>
         </is>
       </c>
       <c r="C7" s="15" t="inlineStr">
         <is>
-          <t>/blog/category/research</t>
+          <t>/blog</t>
         </is>
       </c>
       <c r="D7" s="16" t="inlineStr">
@@ -770,7 +770,7 @@
       </c>
       <c r="G7" s="15" t="inlineStr">
         <is>
-          <t>src/pages/blog/category/[category].astro</t>
+          <t>src/pages/blog/index.astro</t>
         </is>
       </c>
       <c r="H7" s="15" t="inlineStr">
@@ -780,24 +780,24 @@
       </c>
       <c r="I7" s="15" t="inlineStr">
         <is>
-          <t>Category landing for "Research". Dynamic route.</t>
+          <t>Blog landing. Lists all posts with category filter.</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="15" t="inlineStr">
         <is>
-          <t>Blog Category — Insights</t>
+          <t>Blog Category — Research</t>
         </is>
       </c>
       <c r="B8" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/category/insights</t>
+          <t>https://compoundhealth.io/blog/category/research</t>
         </is>
       </c>
       <c r="C8" s="15" t="inlineStr">
         <is>
-          <t>/blog/category/insights</t>
+          <t>/blog/category/research</t>
         </is>
       </c>
       <c r="D8" s="16" t="inlineStr">
@@ -827,24 +827,24 @@
       </c>
       <c r="I8" s="15" t="inlineStr">
         <is>
-          <t>Category landing for "Insights". Dynamic route.</t>
+          <t>Category landing for "Research". Dynamic route.</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="15" t="inlineStr">
         <is>
-          <t>Blog Post — Biomarkers that matter after fifty</t>
+          <t>Blog Category — Insights</t>
         </is>
       </c>
       <c r="B9" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/biomarkers-that-matter-after-fifty</t>
+          <t>https://compoundhealth.io/blog/category/insights</t>
         </is>
       </c>
       <c r="C9" s="15" t="inlineStr">
         <is>
-          <t>/blog/biomarkers-that-matter-after-fifty</t>
+          <t>/blog/category/insights</t>
         </is>
       </c>
       <c r="D9" s="16" t="inlineStr">
@@ -864,7 +864,7 @@
       </c>
       <c r="G9" s="15" t="inlineStr">
         <is>
-          <t>src/pages/blog/[slug].astro</t>
+          <t>src/pages/blog/category/[category].astro</t>
         </is>
       </c>
       <c r="H9" s="15" t="inlineStr">
@@ -874,24 +874,24 @@
       </c>
       <c r="I9" s="15" t="inlineStr">
         <is>
-          <t>Dummy content. Featured post on /blog.</t>
+          <t>Category landing for "Insights". Dynamic route.</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="15" t="inlineStr">
         <is>
-          <t>Blog Post — What VO2 max really tells you</t>
+          <t>Blog Post — Biomarkers that matter after fifty</t>
         </is>
       </c>
       <c r="B10" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/what-vo2-max-really-tells-you</t>
+          <t>https://compoundhealth.io/blog/biomarkers-that-matter-after-fifty</t>
         </is>
       </c>
       <c r="C10" s="15" t="inlineStr">
         <is>
-          <t>/blog/what-vo2-max-really-tells-you</t>
+          <t>/blog/biomarkers-that-matter-after-fifty</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
@@ -921,24 +921,24 @@
       </c>
       <c r="I10" s="15" t="inlineStr">
         <is>
-          <t>Dummy content.</t>
+          <t>Dummy content. Featured post on /blog.</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="15" t="inlineStr">
         <is>
-          <t>Blog Post — Longevity and the family balance sheet</t>
+          <t>Blog Post — What VO2 max really tells you</t>
         </is>
       </c>
       <c r="B11" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/longevity-and-the-family-balance-sheet</t>
+          <t>https://compoundhealth.io/blog/what-vo2-max-really-tells-you</t>
         </is>
       </c>
       <c r="C11" s="15" t="inlineStr">
         <is>
-          <t>/blog/longevity-and-the-family-balance-sheet</t>
+          <t>/blog/what-vo2-max-really-tells-you</t>
         </is>
       </c>
       <c r="D11" s="16" t="inlineStr">
@@ -975,17 +975,17 @@
     <row r="12">
       <c r="A12" s="15" t="inlineStr">
         <is>
-          <t>Blog Post — CGMs for non-diabetics</t>
+          <t>Blog Post — Longevity and the family balance sheet</t>
         </is>
       </c>
       <c r="B12" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/continuous-glucose-monitoring-for-non-diabetics</t>
+          <t>https://compoundhealth.io/blog/longevity-and-the-family-balance-sheet</t>
         </is>
       </c>
       <c r="C12" s="15" t="inlineStr">
         <is>
-          <t>/blog/continuous-glucose-monitoring-for-non-diabetics</t>
+          <t>/blog/longevity-and-the-family-balance-sheet</t>
         </is>
       </c>
       <c r="D12" s="16" t="inlineStr">
@@ -1022,17 +1022,17 @@
     <row r="13">
       <c r="A13" s="15" t="inlineStr">
         <is>
-          <t>Blog Post — Sleep as a biomarker</t>
+          <t>Blog Post — CGMs for non-diabetics</t>
         </is>
       </c>
       <c r="B13" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/sleep-the-biomarker-we-undervalue</t>
+          <t>https://compoundhealth.io/blog/continuous-glucose-monitoring-for-non-diabetics</t>
         </is>
       </c>
       <c r="C13" s="15" t="inlineStr">
         <is>
-          <t>/blog/sleep-the-biomarker-we-undervalue</t>
+          <t>/blog/continuous-glucose-monitoring-for-non-diabetics</t>
         </is>
       </c>
       <c r="D13" s="16" t="inlineStr">
@@ -1069,17 +1069,17 @@
     <row r="14">
       <c r="A14" s="15" t="inlineStr">
         <is>
-          <t>Blog Post — A note on biological age tests</t>
+          <t>Blog Post — Sleep as a biomarker</t>
         </is>
       </c>
       <c r="B14" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/blog/a-note-on-biological-age-tests</t>
+          <t>https://compoundhealth.io/blog/sleep-the-biomarker-we-undervalue</t>
         </is>
       </c>
       <c r="C14" s="15" t="inlineStr">
         <is>
-          <t>/blog/a-note-on-biological-age-tests</t>
+          <t>/blog/sleep-the-biomarker-we-undervalue</t>
         </is>
       </c>
       <c r="D14" s="16" t="inlineStr">
@@ -1116,17 +1116,17 @@
     <row r="15">
       <c r="A15" s="15" t="inlineStr">
         <is>
-          <t>Author — Imogen Asher</t>
+          <t>Blog Post — A note on biological age tests</t>
         </is>
       </c>
       <c r="B15" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/authors/imogen-asher</t>
+          <t>https://compoundhealth.io/blog/a-note-on-biological-age-tests</t>
         </is>
       </c>
       <c r="C15" s="15" t="inlineStr">
         <is>
-          <t>/authors/imogen-asher</t>
+          <t>/blog/a-note-on-biological-age-tests</t>
         </is>
       </c>
       <c r="D15" s="16" t="inlineStr">
@@ -1146,7 +1146,7 @@
       </c>
       <c r="G15" s="15" t="inlineStr">
         <is>
-          <t>src/pages/authors/[author].astro</t>
+          <t>src/pages/blog/[slug].astro</t>
         </is>
       </c>
       <c r="H15" s="15" t="inlineStr">
@@ -1156,24 +1156,24 @@
       </c>
       <c r="I15" s="15" t="inlineStr">
         <is>
-          <t>Dummy author. Posts listed via shared data file.</t>
+          <t>Dummy content.</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="15" t="inlineStr">
         <is>
-          <t>Author — Henry Cavendish</t>
+          <t>Author — Imogen Asher</t>
         </is>
       </c>
       <c r="B16" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/authors/henry-cavendish</t>
+          <t>https://compoundhealth.io/authors/imogen-asher</t>
         </is>
       </c>
       <c r="C16" s="15" t="inlineStr">
         <is>
-          <t>/authors/henry-cavendish</t>
+          <t>/authors/imogen-asher</t>
         </is>
       </c>
       <c r="D16" s="16" t="inlineStr">
@@ -1210,17 +1210,17 @@
     <row r="17">
       <c r="A17" s="15" t="inlineStr">
         <is>
-          <t>Design System — Overview</t>
+          <t>Author — Henry Cavendish</t>
         </is>
       </c>
       <c r="B17" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/design-system</t>
+          <t>https://compoundhealth.io/authors/henry-cavendish</t>
         </is>
       </c>
       <c r="C17" s="15" t="inlineStr">
         <is>
-          <t>/design-system</t>
+          <t>/authors/henry-cavendish</t>
         </is>
       </c>
       <c r="D17" s="16" t="inlineStr">
@@ -1235,12 +1235,12 @@
       </c>
       <c r="F17" s="15" t="inlineStr">
         <is>
-          <t>DesignSystemLayout</t>
+          <t>BlogLayout</t>
         </is>
       </c>
       <c r="G17" s="15" t="inlineStr">
         <is>
-          <t>src/pages/design-system/index.astro</t>
+          <t>src/pages/authors/[author].astro</t>
         </is>
       </c>
       <c r="H17" s="15" t="inlineStr">
@@ -1250,24 +1250,24 @@
       </c>
       <c r="I17" s="15" t="inlineStr">
         <is>
-          <t>Internal design system overview. Atomic methodology + Finsweet Client-First naming.</t>
+          <t>Dummy author. Posts listed via shared data file.</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="15" t="inlineStr">
         <is>
-          <t>Design System — Atoms</t>
+          <t>Design System — Overview</t>
         </is>
       </c>
       <c r="B18" s="15" t="inlineStr">
         <is>
-          <t>https://compoundhealth.io/design-system/atoms</t>
+          <t>https://compoundhealth.io/design-system</t>
         </is>
       </c>
       <c r="C18" s="15" t="inlineStr">
         <is>
-          <t>/design-system/atoms</t>
+          <t>/design-system</t>
         </is>
       </c>
       <c r="D18" s="16" t="inlineStr">
@@ -1287,7 +1287,7 @@
       </c>
       <c r="G18" s="15" t="inlineStr">
         <is>
-          <t>src/pages/design-system/atoms.astro</t>
+          <t>src/pages/design-system/index.astro</t>
         </is>
       </c>
       <c r="H18" s="15" t="inlineStr">
@@ -1297,52 +1297,99 @@
       </c>
       <c r="I18" s="15" t="inlineStr">
         <is>
-          <t>Colour, typography, spacing, radii, buttons, badges, eyebrows, dots, avatars, dividers, inputs, links, motion.</t>
+          <t>Internal design system overview. Atomic methodology + Finsweet Client-First naming.</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="15" t="inlineStr">
         <is>
+          <t>Design System — Atoms</t>
+        </is>
+      </c>
+      <c r="B19" s="15" t="inlineStr">
+        <is>
+          <t>https://compoundhealth.io/design-system/atoms</t>
+        </is>
+      </c>
+      <c r="C19" s="15" t="inlineStr">
+        <is>
+          <t>/design-system/atoms</t>
+        </is>
+      </c>
+      <c r="D19" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>Noindex</t>
+        </is>
+      </c>
+      <c r="F19" s="15" t="inlineStr">
+        <is>
+          <t>DesignSystemLayout</t>
+        </is>
+      </c>
+      <c r="G19" s="15" t="inlineStr">
+        <is>
+          <t>src/pages/design-system/atoms.astro</t>
+        </is>
+      </c>
+      <c r="H19" s="15" t="inlineStr">
+        <is>
+          <t>2026-06-02</t>
+        </is>
+      </c>
+      <c r="I19" s="15" t="inlineStr">
+        <is>
+          <t>Colour, typography, spacing, radii, buttons, badges, eyebrows, dots, avatars, dividers, inputs, links, motion.</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="15" t="inlineStr">
+        <is>
           <t>Design System — Molecules</t>
         </is>
       </c>
-      <c r="B19" s="15" t="inlineStr">
+      <c r="B20" s="15" t="inlineStr">
         <is>
           <t>https://compoundhealth.io/design-system/molecules</t>
         </is>
       </c>
-      <c r="C19" s="15" t="inlineStr">
+      <c r="C20" s="15" t="inlineStr">
         <is>
           <t>/design-system/molecules</t>
         </is>
       </c>
-      <c r="D19" s="16" t="inlineStr">
-        <is>
-          <t>Live</t>
-        </is>
-      </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="D20" s="16" t="inlineStr">
+        <is>
+          <t>Live</t>
+        </is>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>Noindex</t>
         </is>
       </c>
-      <c r="F19" s="15" t="inlineStr">
+      <c r="F20" s="15" t="inlineStr">
         <is>
           <t>DesignSystemLayout</t>
         </is>
       </c>
-      <c r="G19" s="15" t="inlineStr">
+      <c r="G20" s="15" t="inlineStr">
         <is>
           <t>src/pages/design-system/molecules.astro</t>
         </is>
       </c>
-      <c r="H19" s="15" t="inlineStr">
+      <c r="H20" s="15" t="inlineStr">
         <is>
           <t>2026-06-02</t>
         </is>
       </c>
-      <c r="I19" s="15" t="inlineStr">
+      <c r="I20" s="15" t="inlineStr">
         <is>
           <t>Step, plan, testimonial, credibility, metric, case stat, case quote, speaker, form field, mobile menu link, author chip, author stack, post card, tag group, breadcrumb, author panel.</t>
         </is>

</xml_diff>